<commit_message>
Add new temporary Excel file for Week 1 analysis
</commit_message>
<xml_diff>
--- a/week_1/Synthetic Data.xlsx
+++ b/week_1/Synthetic Data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Uyanwune chekwube\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Uyanwune chekwube\Downloads\CreditRiskAnalysis\week_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="240">
   <si>
     <t>signup_date</t>
   </si>
@@ -747,6 +747,12 @@
   </si>
   <si>
     <t>cumulative_paid</t>
+  </si>
+  <si>
+    <t>Installments</t>
+  </si>
+  <si>
+    <t>None</t>
   </si>
 </sst>
 </file>
@@ -785,12 +791,30 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -806,7 +830,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -846,6 +870,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3356,10 +3385,10 @@
     <col min="4" max="4" width="17.36328125" style="6" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.453125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.1796875" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.36328125" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.7265625" style="6" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.26953125" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.36328125" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.26953125" style="6" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="14.90625" style="6" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="15.36328125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="22.1796875" bestFit="1" customWidth="1"/>
@@ -3565,7 +3594,7 @@
         <v>226</v>
       </c>
       <c r="K5" s="7">
-        <f>E5*F5*H5+G5+E5</f>
+        <f t="shared" ref="K5:K21" si="1">E5*F5*H5+G5+E5</f>
         <v>126200</v>
       </c>
     </row>
@@ -3602,7 +3631,7 @@
         <v>226</v>
       </c>
       <c r="K6" s="7">
-        <f>E6*F6*H6+G6+E6</f>
+        <f t="shared" si="1"/>
         <v>148600</v>
       </c>
     </row>
@@ -3639,7 +3668,7 @@
         <v>227</v>
       </c>
       <c r="K7" s="7">
-        <f>E7*F7*H7+G7+E7</f>
+        <f t="shared" si="1"/>
         <v>173000</v>
       </c>
     </row>
@@ -3676,7 +3705,7 @@
         <v>224</v>
       </c>
       <c r="K8" s="7">
-        <f>E8*F8*H8+G8+E8</f>
+        <f t="shared" si="1"/>
         <v>192900</v>
       </c>
     </row>
@@ -3713,7 +3742,7 @@
         <v>224</v>
       </c>
       <c r="K9" s="7">
-        <f>E9*F9*H9+G9+E9</f>
+        <f t="shared" si="1"/>
         <v>68200</v>
       </c>
       <c r="L9">
@@ -3754,7 +3783,7 @@
         <v>226</v>
       </c>
       <c r="K10" s="7">
-        <f>E10*F10*H10+G10+E10</f>
+        <f t="shared" si="1"/>
         <v>91600</v>
       </c>
     </row>
@@ -3791,7 +3820,7 @@
         <v>228</v>
       </c>
       <c r="K11" s="7">
-        <f>E11*F11*H11+G11+E11</f>
+        <f t="shared" si="1"/>
         <v>115000</v>
       </c>
     </row>
@@ -3828,7 +3857,7 @@
         <v>226</v>
       </c>
       <c r="K12" s="7">
-        <f>E12*F12*H12+G12+E12</f>
+        <f t="shared" si="1"/>
         <v>137400</v>
       </c>
     </row>
@@ -3865,7 +3894,7 @@
         <v>224</v>
       </c>
       <c r="K13" s="7">
-        <f>E13*F13*H13+G13+E13</f>
+        <f t="shared" si="1"/>
         <v>159800</v>
       </c>
     </row>
@@ -3902,7 +3931,7 @@
         <v>226</v>
       </c>
       <c r="K14" s="7">
-        <f>E14*F14*H14+G14+E14</f>
+        <f t="shared" si="1"/>
         <v>184200</v>
       </c>
     </row>
@@ -3939,7 +3968,7 @@
         <v>228</v>
       </c>
       <c r="K15" s="7">
-        <f>E15*F15*H15+G15+E15</f>
+        <f t="shared" si="1"/>
         <v>206600</v>
       </c>
     </row>
@@ -3976,7 +4005,7 @@
         <v>228</v>
       </c>
       <c r="K16" s="7">
-        <f>E16*F16*H16+G16+E16</f>
+        <f t="shared" si="1"/>
         <v>229000</v>
       </c>
     </row>
@@ -4013,7 +4042,7 @@
         <v>229</v>
       </c>
       <c r="K17" s="7">
-        <f>E17*F17*H17+G17+E17</f>
+        <f t="shared" si="1"/>
         <v>80400</v>
       </c>
     </row>
@@ -4050,7 +4079,7 @@
         <v>229</v>
       </c>
       <c r="K18" s="7">
-        <f>E18*F18*H18+G18+E18</f>
+        <f t="shared" si="1"/>
         <v>102800</v>
       </c>
     </row>
@@ -4087,7 +4116,7 @@
         <v>225</v>
       </c>
       <c r="K19" s="7">
-        <f>E19*F19*H19+G19+E19</f>
+        <f t="shared" si="1"/>
         <v>126200</v>
       </c>
     </row>
@@ -4124,7 +4153,7 @@
         <v>224</v>
       </c>
       <c r="K20" s="7">
-        <f>E20*F20*H20+G20+E20</f>
+        <f t="shared" si="1"/>
         <v>57000</v>
       </c>
     </row>
@@ -4161,8 +4190,13 @@
         <v>227</v>
       </c>
       <c r="K21" s="7">
-        <f>E21*F21*H21+G21+E21</f>
+        <f t="shared" si="1"/>
         <v>85000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="B23" s="17" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.35">
@@ -4215,7 +4249,23 @@
         <f>K2/H2</f>
         <v>19000</v>
       </c>
-      <c r="H25" s="16"/>
+      <c r="F25" t="s">
+        <v>66</v>
+      </c>
+      <c r="G25" s="13">
+        <v>45933</v>
+      </c>
+      <c r="H25" s="16">
+        <f>SUMIFS(D25:D27, A25:A27,F25, C25:C27, "&lt;="&amp;C27)</f>
+        <v>57000</v>
+      </c>
+      <c r="I25" s="6">
+        <f>SUMIFS(D25:D27, A25:A27,F25, C25:C27, "&lt;="&amp;C27)</f>
+        <v>57000</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>239</v>
+      </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
@@ -4261,6 +4311,20 @@
         <f>K3/H3</f>
         <v>27133.333333333332</v>
       </c>
+      <c r="G28" s="13">
+        <v>45964</v>
+      </c>
+      <c r="H28" s="6">
+        <f>SUMIFS(D28:D30, A28:A30,A3,C28:C30,"&lt;="&amp;C30)</f>
+        <v>81400</v>
+      </c>
+      <c r="I28" s="6">
+        <f>SUMIFS(D28:D30, A28:A30,A3,C28:C30,"&lt;="&amp;C30)</f>
+        <v>81400</v>
+      </c>
+      <c r="J28" s="18" t="s">
+        <v>239</v>
+      </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
@@ -4322,7 +4386,7 @@
         <v>32666.666666666668</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>72</v>
       </c>
@@ -4333,11 +4397,23 @@
         <v>45935</v>
       </c>
       <c r="D33" s="6">
-        <f>K4/H4</f>
+        <f>D32</f>
         <v>32666.666666666668</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H33" s="6">
+        <f>SUMIFS(D31:D33, A31:A33, A4, C31:C33, "&lt;="&amp;C33)</f>
+        <v>98000</v>
+      </c>
+      <c r="I33" s="6">
+        <f>SUMIFS(D31:D32,A31:A32, A4,C31:C32, "&lt;="&amp;C32)</f>
+        <v>65333.333333333336</v>
+      </c>
+      <c r="J33" s="19">
+        <f>MAX(0,H33-I33)</f>
+        <v>32666.666666666664</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>74</v>
       </c>
@@ -4352,7 +4428,7 @@
         <v>42066.666666666664</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>74</v>
       </c>
@@ -4367,7 +4443,7 @@
         <v>42066.666666666664</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>74</v>
       </c>
@@ -4382,62 +4458,83 @@
         <v>42066.666666666664</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+      <c r="B37" s="2">
+        <v>1</v>
+      </c>
+      <c r="D37" s="6">
+        <f>K6/H6</f>
+        <v>49533.333333333336</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+      <c r="B38" s="2">
+        <v>2</v>
+      </c>
+      <c r="D38" s="6">
+        <f>K6/H5</f>
+        <v>49533.333333333336</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+      <c r="B39" s="2">
+        <v>3</v>
+      </c>
+      <c r="D39" s="6">
+        <f>K6/H6</f>
+        <v>49533.333333333336</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>203</v>
       </c>

</xml_diff>

<commit_message>
Update Synthetic Data.xlsx for Week 1 analysis
</commit_message>
<xml_diff>
--- a/week_1/Synthetic Data.xlsx
+++ b/week_1/Synthetic Data.xlsx
@@ -830,7 +830,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -875,6 +875,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4252,9 +4253,7 @@
       <c r="F25" t="s">
         <v>66</v>
       </c>
-      <c r="G25" s="13">
-        <v>45933</v>
-      </c>
+      <c r="G25" s="13"/>
       <c r="H25" s="16">
         <f>SUMIFS(D25:D27, A25:A27,F25, C25:C27, "&lt;="&amp;C27)</f>
         <v>57000</v>
@@ -4263,7 +4262,7 @@
         <f>SUMIFS(D25:D27, A25:A27,F25, C25:C27, "&lt;="&amp;C27)</f>
         <v>57000</v>
       </c>
-      <c r="J25" s="6" t="s">
+      <c r="J25" s="20" t="s">
         <v>239</v>
       </c>
     </row>
@@ -4311,9 +4310,7 @@
         <f>K3/H3</f>
         <v>27133.333333333332</v>
       </c>
-      <c r="G28" s="13">
-        <v>45964</v>
-      </c>
+      <c r="G28" s="13"/>
       <c r="H28" s="6">
         <f>SUMIFS(D28:D30, A28:A30,A3,C28:C30,"&lt;="&amp;C30)</f>
         <v>81400</v>
@@ -4386,7 +4383,7 @@
         <v>32666.666666666668</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>72</v>
       </c>
@@ -4405,15 +4402,19 @@
         <v>98000</v>
       </c>
       <c r="I33" s="6">
-        <f>SUMIFS(D31:D32,A31:A32, A4,C31:C32, "&lt;="&amp;C32)</f>
+        <f>SUMIFS(D31:D32,A31:A32, A4,C31:C32, "&lt;="&amp;C33)</f>
         <v>65333.333333333336</v>
       </c>
       <c r="J33" s="19">
         <f>MAX(0,H33-I33)</f>
         <v>32666.666666666664</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K33" s="13">
+        <f>C33</f>
+        <v>45935</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>74</v>
       </c>
@@ -4428,7 +4429,7 @@
         <v>42066.666666666664</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>74</v>
       </c>
@@ -4443,7 +4444,7 @@
         <v>42066.666666666664</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>74</v>
       </c>
@@ -4458,7 +4459,7 @@
         <v>42066.666666666664</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>76</v>
       </c>
@@ -4470,7 +4471,7 @@
         <v>49533.333333333336</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>76</v>
       </c>
@@ -4482,7 +4483,7 @@
         <v>49533.333333333336</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>76</v>
       </c>
@@ -4494,47 +4495,47 @@
         <v>49533.333333333336</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>203</v>
       </c>

</xml_diff>